<commit_message>
traitement comment sur logicalID
suite au traitement du commentaire https://github.com/ansforge/IG-FHIR-PDSM4DMP-EEDS/pull/16/changes#r4025909803, mise en cohérence de l'IG avec utilisation de Claude 6903b53a8c3010746b8a4cdb2873549814d0d0fb
</commit_message>
<xml_diff>
--- a/add-mapping-xds-fhir/ig/StructureDefinition-DocumentEntry.xlsx
+++ b/add-mapping-xds-fhir/ig/StructureDefinition-DocumentEntry.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-22T15:20:18+00:00</t>
+    <t>2026-09-22T17:31:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -263,7 +263,7 @@
     <t>Identifiant unique affecté à la version de la fiche référençant le document.</t>
   </si>
   <si>
-    <t>Les valeurs possibles pour cette métadonnée doivent être un code provenant du jeu de valeurs mis à disposition par le projet. En l’absence de spécifications complémentaires, le jeu de valeurs JDV_J52_AvailabilityStatus_CISIS peut être utilisé.</t>
+    <t>Cet identifiant est attribué par le registre du système cible lors de la soumission. Il change à chaque nouvelle version de la fiche, à la différence de logicalId qui reste invariable.</t>
   </si>
   <si>
     <t>DocumentEntry.logicalId</t>

</xml_diff>